<commit_message>
Add 3 new students (DADIREDDI VARSHITHA, V MALLIKARJUNA, BOMMADI ISHANT SRI) bringing total DB count to 262 and update Excel sheets
</commit_message>
<xml_diff>
--- a/CSI_KARE_ML_Pipeline_All_Registrations_Clean.xlsx
+++ b/CSI_KARE_ML_Pipeline_All_Registrations_Clean.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="All Participants" sheetId="1" r:id="rId1"/>
+    <sheet name="All Registrations" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P260"/>
+  <dimension ref="A1:P263"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -1911,7 +1911,7 @@
         <v>claim-group-3/payment-screenshots/99240040422</v>
       </c>
       <c r="O30" t="str">
-        <v>[Base64 Screenshot Attached]</v>
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/99240040422.jpg</v>
       </c>
       <c r="P30" t="str">
         <v>7/8/2026, 9:41:59 am</v>
@@ -2161,7 +2161,7 @@
         <v>claim-group-3/payment-screenshots/99240040597</v>
       </c>
       <c r="O35" t="str">
-        <v>[Base64 Screenshot Attached]</v>
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/99240040597.jpg</v>
       </c>
       <c r="P35" t="str">
         <v>7/8/2026, 9:43:21 am</v>
@@ -5525,7 +5525,7 @@
         <v>MANUKINDA KRISHNAVAMSI</v>
       </c>
       <c r="C103" t="str">
-        <v>999240040148</v>
+        <v>99240040148</v>
       </c>
       <c r="D103" t="str">
         <v>T2608070952318053181777/ 067644050887</v>
@@ -6261,7 +6261,7 @@
         <v>claim-group-3/payment-screenshots/99240040084</v>
       </c>
       <c r="O117" t="str">
-        <v>[Base64 Screenshot Attached]</v>
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/99240040084.jpg</v>
       </c>
       <c r="P117" t="str">
         <v>7/8/2026, 9:55:12 am</v>
@@ -7361,7 +7361,7 @@
         <v>claim-group-3/payment-screenshots/99240040064</v>
       </c>
       <c r="O139" t="str">
-        <v>[Base64 Screenshot Attached]</v>
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/99240040064.jpg</v>
       </c>
       <c r="P139" t="str">
         <v>7/8/2026, 9:56:53 am</v>
@@ -7511,7 +7511,7 @@
         <v>claim-group-3/payment-screenshots/99240040598</v>
       </c>
       <c r="O142" t="str">
-        <v>[Base64 Screenshot Attached]</v>
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/99240040598.jpg</v>
       </c>
       <c r="P142" t="str">
         <v>7/8/2026, 9:57:04 am</v>
@@ -7661,7 +7661,7 @@
         <v>claim-group-3/payment-screenshots/99240041425</v>
       </c>
       <c r="O145" t="str">
-        <v>[Base64 Screenshot Attached]</v>
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/99240041425.jpg</v>
       </c>
       <c r="P145" t="str">
         <v>7/8/2026, 9:57:28 am</v>
@@ -8108,10 +8108,10 @@
         <v/>
       </c>
       <c r="N154" t="str">
-        <v>claim-group-3/payment-screenshots/claim-group-3/payment-screenshots/99240041034</v>
+        <v>claim-group-3/payment-screenshots/99240041034</v>
       </c>
       <c r="O154" t="str">
-        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/claim-group-3/payment-screenshots/99240041034.jpg</v>
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/99240041034.jpg</v>
       </c>
       <c r="P154" t="str">
         <v>7/8/2026, 9:57:59 am</v>
@@ -8311,7 +8311,7 @@
         <v>claim-group-3/payment-screenshots/99240041336</v>
       </c>
       <c r="O158" t="str">
-        <v>[Base64 Screenshot Attached]</v>
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/99240041336.jpg</v>
       </c>
       <c r="P158" t="str">
         <v>7/8/2026, 9:58:05 am</v>
@@ -8911,7 +8911,7 @@
         <v>claim-group-3/payment-screenshots/99240040598</v>
       </c>
       <c r="O170" t="str">
-        <v>[Base64 Screenshot Attached]</v>
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/99240040598.jpg</v>
       </c>
       <c r="P170" t="str">
         <v>7/8/2026, 9:58:45 am</v>
@@ -9161,7 +9161,7 @@
         <v>claim-group-3/payment-screenshots/99240040017</v>
       </c>
       <c r="O175" t="str">
-        <v>[Base64 Screenshot Attached]</v>
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/99240040017.jpg</v>
       </c>
       <c r="P175" t="str">
         <v>7/8/2026, 9:58:55 am</v>
@@ -10261,7 +10261,7 @@
         <v>claim-group-3/payment-screenshots/99240041323</v>
       </c>
       <c r="O197" t="str">
-        <v>[Base64 Screenshot Attached]</v>
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/99240041323.jpg</v>
       </c>
       <c r="P197" t="str">
         <v>7/8/2026, 10:01:26 am</v>
@@ -10361,7 +10361,7 @@
         <v>claim-group-3/payment-screenshots/99240040713</v>
       </c>
       <c r="O199" t="str">
-        <v>[Base64 Screenshot Attached]</v>
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/99240040713.jpg</v>
       </c>
       <c r="P199" t="str">
         <v>7/8/2026, 10:01:35 am</v>
@@ -10761,7 +10761,7 @@
         <v>claim-group-3/payment-screenshots/99240041315</v>
       </c>
       <c r="O207" t="str">
-        <v>[Base64 Screenshot Attached]</v>
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/99240041315.jpg</v>
       </c>
       <c r="P207" t="str">
         <v>7/8/2026, 10:02:17 am</v>
@@ -10811,7 +10811,7 @@
         <v>claim-group-3/payment-screenshots/99240040321</v>
       </c>
       <c r="O208" t="str">
-        <v>[Base64 Screenshot Attached]</v>
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/99240040321.jpg</v>
       </c>
       <c r="P208" t="str">
         <v>7/8/2026, 10:02:21 am</v>
@@ -11108,10 +11108,10 @@
         <v/>
       </c>
       <c r="N214" t="str">
-        <v>claim-group-3/payment-screenshots/claim-group-3/payment-screenshots/99240041002</v>
+        <v>claim-group-3/payment-screenshots/99240041002</v>
       </c>
       <c r="O214" t="str">
-        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786077169/claim-group-3/payment-screenshots/claim-group-3/payment-screenshots/99240041002.jpg</v>
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/99240041002.jpg</v>
       </c>
       <c r="P214" t="str">
         <v>7/8/2026, 10:02:50 am</v>
@@ -12011,7 +12011,7 @@
         <v>claim-group-3/payment-screenshots/99240040688</v>
       </c>
       <c r="O232" t="str">
-        <v>[Base64 Screenshot Attached]</v>
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/99240040688.jpg</v>
       </c>
       <c r="P232" t="str">
         <v>7/8/2026, 10:09:57 am</v>
@@ -12111,7 +12111,7 @@
         <v>claim-group-3/payment-screenshots/99240040666</v>
       </c>
       <c r="O234" t="str">
-        <v>https://images.unsplash.com/photo-1554224155-8d04cb21cd6c?w=400&amp;q=80</v>
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/99240040666.jpg</v>
       </c>
       <c r="P234" t="str">
         <v>7/8/2026, 12:35:22 pm</v>
@@ -12161,7 +12161,7 @@
         <v>claim-group-3/payment-screenshots/99240040388</v>
       </c>
       <c r="O235" t="str">
-        <v>https://images.unsplash.com/photo-1554224155-8d04cb21cd6c?w=400&amp;q=80</v>
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/99240040388.jpg</v>
       </c>
       <c r="P235" t="str">
         <v>7/8/2026, 12:35:23 pm</v>
@@ -12211,7 +12211,7 @@
         <v>claim-group-3/payment-screenshots/9924005417</v>
       </c>
       <c r="O236" t="str">
-        <v>https://images.unsplash.com/photo-1554224155-8d04cb21cd6c?w=400&amp;q=80</v>
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/9924005417.jpg</v>
       </c>
       <c r="P236" t="str">
         <v>7/8/2026, 12:35:24 pm</v>
@@ -12261,7 +12261,7 @@
         <v>claim-group-3/payment-screenshots/99240040616</v>
       </c>
       <c r="O237" t="str">
-        <v>https://images.unsplash.com/photo-1554224155-8d04cb21cd6c?w=400&amp;q=80</v>
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/99240040616.jpg</v>
       </c>
       <c r="P237" t="str">
         <v>7/8/2026, 12:35:24 pm</v>
@@ -12311,7 +12311,7 @@
         <v>claim-group-3/payment-screenshots/99240040701</v>
       </c>
       <c r="O238" t="str">
-        <v>https://images.unsplash.com/photo-1554224155-8d04cb21cd6c?w=400&amp;q=80</v>
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/99240040701.jpg</v>
       </c>
       <c r="P238" t="str">
         <v>7/8/2026, 12:35:24 pm</v>
@@ -12361,7 +12361,7 @@
         <v>claim-group-3/payment-screenshots/99240040794</v>
       </c>
       <c r="O239" t="str">
-        <v>https://images.unsplash.com/photo-1554224155-8d04cb21cd6c?w=400&amp;q=80</v>
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/99240040794.jpg</v>
       </c>
       <c r="P239" t="str">
         <v>7/8/2026, 12:35:25 pm</v>
@@ -12411,7 +12411,7 @@
         <v>claim-group-3/payment-screenshots/99240040139</v>
       </c>
       <c r="O240" t="str">
-        <v>https://images.unsplash.com/photo-1554224155-8d04cb21cd6c?w=400&amp;q=80</v>
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/99240040139.jpg</v>
       </c>
       <c r="P240" t="str">
         <v>7/8/2026, 12:35:25 pm</v>
@@ -12461,7 +12461,7 @@
         <v>claim-group-3/payment-screenshots/9924008099</v>
       </c>
       <c r="O241" t="str">
-        <v>https://images.unsplash.com/photo-1554224155-8d04cb21cd6c?w=400&amp;q=80</v>
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/9924008099.jpg</v>
       </c>
       <c r="P241" t="str">
         <v>7/8/2026, 12:35:25 pm</v>
@@ -12511,7 +12511,7 @@
         <v>claim-group-3/payment-screenshots/99240040214</v>
       </c>
       <c r="O242" t="str">
-        <v>https://images.unsplash.com/photo-1554224155-8d04cb21cd6c?w=400&amp;q=80</v>
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/99240040214.jpg</v>
       </c>
       <c r="P242" t="str">
         <v>7/8/2026, 12:35:26 pm</v>
@@ -12561,7 +12561,7 @@
         <v>claim-group-3/payment-screenshots/99240041153</v>
       </c>
       <c r="O243" t="str">
-        <v>https://images.unsplash.com/photo-1554224155-8d04cb21cd6c?w=400&amp;q=80</v>
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/99240041153.jpg</v>
       </c>
       <c r="P243" t="str">
         <v>7/8/2026, 12:35:26 pm</v>
@@ -12611,7 +12611,7 @@
         <v>claim-group-3/payment-screenshots/99240041098</v>
       </c>
       <c r="O244" t="str">
-        <v>https://images.unsplash.com/photo-1554224155-8d04cb21cd6c?w=400&amp;q=80</v>
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/99240041098.jpg</v>
       </c>
       <c r="P244" t="str">
         <v>7/8/2026, 12:35:26 pm</v>
@@ -12661,7 +12661,7 @@
         <v>claim-group-3/payment-screenshots/99240040130</v>
       </c>
       <c r="O245" t="str">
-        <v>https://images.unsplash.com/photo-1554224155-8d04cb21cd6c?w=400&amp;q=80</v>
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/99240040130.jpg</v>
       </c>
       <c r="P245" t="str">
         <v>7/8/2026, 12:35:27 pm</v>
@@ -12711,7 +12711,7 @@
         <v>claim-group-3/payment-screenshots/99240040867</v>
       </c>
       <c r="O246" t="str">
-        <v>https://images.unsplash.com/photo-1554224155-8d04cb21cd6c?w=400&amp;q=80</v>
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/99240040867.jpg</v>
       </c>
       <c r="P246" t="str">
         <v>7/8/2026, 12:35:27 pm</v>
@@ -12761,7 +12761,7 @@
         <v>claim-group-3/payment-screenshots/99240040529</v>
       </c>
       <c r="O247" t="str">
-        <v>https://images.unsplash.com/photo-1554224155-8d04cb21cd6c?w=400&amp;q=80</v>
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/99240040529.jpg</v>
       </c>
       <c r="P247" t="str">
         <v>7/8/2026, 12:35:28 pm</v>
@@ -12811,7 +12811,7 @@
         <v>claim-group-3/payment-screenshots/99240041156</v>
       </c>
       <c r="O248" t="str">
-        <v>https://images.unsplash.com/photo-1554224155-8d04cb21cd6c?w=400&amp;q=80</v>
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/99240041156.jpg</v>
       </c>
       <c r="P248" t="str">
         <v>7/8/2026, 12:35:28 pm</v>
@@ -12861,7 +12861,7 @@
         <v>claim-group-3/payment-screenshots/99240041338</v>
       </c>
       <c r="O249" t="str">
-        <v>https://images.unsplash.com/photo-1554224155-8d04cb21cd6c?w=400&amp;q=80</v>
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/99240041338.jpg</v>
       </c>
       <c r="P249" t="str">
         <v>7/8/2026, 12:35:28 pm</v>
@@ -12911,7 +12911,7 @@
         <v>claim-group-3/payment-screenshots/99240040240</v>
       </c>
       <c r="O250" t="str">
-        <v>https://images.unsplash.com/photo-1554224155-8d04cb21cd6c?w=400&amp;q=80</v>
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/99240040240.jpg</v>
       </c>
       <c r="P250" t="str">
         <v>7/8/2026, 12:35:29 pm</v>
@@ -12961,7 +12961,7 @@
         <v>claim-group-3/payment-screenshots/99240041164</v>
       </c>
       <c r="O251" t="str">
-        <v>https://images.unsplash.com/photo-1554224155-8d04cb21cd6c?w=400&amp;q=80</v>
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/99240041164.jpg</v>
       </c>
       <c r="P251" t="str">
         <v>7/8/2026, 12:35:29 pm</v>
@@ -13011,7 +13011,7 @@
         <v>claim-group-3/payment-screenshots/99240040717</v>
       </c>
       <c r="O252" t="str">
-        <v>https://images.unsplash.com/photo-1554224155-8d04cb21cd6c?w=400&amp;q=80</v>
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/99240040717.jpg</v>
       </c>
       <c r="P252" t="str">
         <v>7/8/2026, 12:35:29 pm</v>
@@ -13061,7 +13061,7 @@
         <v>claim-group-3/payment-screenshots/99240040324</v>
       </c>
       <c r="O253" t="str">
-        <v>https://images.unsplash.com/photo-1554224155-8d04cb21cd6c?w=400&amp;q=80</v>
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/99240040324.jpg</v>
       </c>
       <c r="P253" t="str">
         <v>7/8/2026, 12:35:45 pm</v>
@@ -13111,7 +13111,7 @@
         <v>claim-group-3/payment-screenshots/99240040704</v>
       </c>
       <c r="O254" t="str">
-        <v>https://images.unsplash.com/photo-1554224155-8d04cb21cd6c?w=400&amp;q=80</v>
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/99240040704.jpg</v>
       </c>
       <c r="P254" t="str">
         <v>7/8/2026, 12:35:45 pm</v>
@@ -13161,7 +13161,7 @@
         <v>claim-group-3/payment-screenshots/99240040502</v>
       </c>
       <c r="O255" t="str">
-        <v>https://images.unsplash.com/photo-1554224155-8d04cb21cd6c?w=400&amp;q=80</v>
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/99240040502.jpg</v>
       </c>
       <c r="P255" t="str">
         <v>7/8/2026, 12:35:46 pm</v>
@@ -13211,7 +13211,7 @@
         <v>claim-group-3/payment-screenshots/99230040331</v>
       </c>
       <c r="O256" t="str">
-        <v>https://images.unsplash.com/photo-1554224155-8d04cb21cd6c?w=400&amp;q=80</v>
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/99230040331.jpg</v>
       </c>
       <c r="P256" t="str">
         <v>7/8/2026, 12:35:46 pm</v>
@@ -13261,7 +13261,7 @@
         <v>claim-group-3/payment-screenshots/99240040070</v>
       </c>
       <c r="O257" t="str">
-        <v>https://images.unsplash.com/photo-1554224155-8d04cb21cd6c?w=400&amp;q=80</v>
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/99240040070.jpg</v>
       </c>
       <c r="P257" t="str">
         <v>7/8/2026, 12:35:46 pm</v>
@@ -13311,7 +13311,7 @@
         <v>claim-group-3/payment-screenshots/99240040668</v>
       </c>
       <c r="O258" t="str">
-        <v>https://images.unsplash.com/photo-1554224155-8d04cb21cd6c?w=400&amp;q=80</v>
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/99240040668.jpg</v>
       </c>
       <c r="P258" t="str">
         <v>7/8/2026, 12:35:47 pm</v>
@@ -13361,7 +13361,7 @@
         <v>claim-group-3/payment-screenshots/99240010723</v>
       </c>
       <c r="O259" t="str">
-        <v>https://images.unsplash.com/photo-1554224155-8d04cb21cd6c?w=400&amp;q=80</v>
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/99240010723.jpg</v>
       </c>
       <c r="P259" t="str">
         <v>7/8/2026, 12:35:47 pm</v>
@@ -13411,15 +13411,165 @@
         <v>claim-group-3/payment-screenshots/99240040304</v>
       </c>
       <c r="O260" t="str">
-        <v>https://images.unsplash.com/photo-1554224155-8d04cb21cd6c?w=400&amp;q=80</v>
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/99240040304.jpg</v>
       </c>
       <c r="P260" t="str">
         <v>7/8/2026, 12:35:48 pm</v>
       </c>
     </row>
+    <row r="261">
+      <c r="A261">
+        <v>260</v>
+      </c>
+      <c r="B261" t="str">
+        <v>DADIREDDI VARSHITHA</v>
+      </c>
+      <c r="C261" t="str">
+        <v>99240040687</v>
+      </c>
+      <c r="D261" t="str">
+        <v>154036284158</v>
+      </c>
+      <c r="E261" t="str">
+        <v>99240040687@klu.ac.in</v>
+      </c>
+      <c r="F261" t="str">
+        <v>9876543210</v>
+      </c>
+      <c r="G261" t="str">
+        <v>CSE</v>
+      </c>
+      <c r="H261" t="str">
+        <v>III Year</v>
+      </c>
+      <c r="I261" t="str">
+        <v>24S08</v>
+      </c>
+      <c r="J261" t="str">
+        <v>Hosteller</v>
+      </c>
+      <c r="K261" t="str">
+        <v>Approved</v>
+      </c>
+      <c r="L261" t="str">
+        <v>Registered</v>
+      </c>
+      <c r="M261" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="N261" t="str">
+        <v>claim-group-3/payment-screenshots/99240040687</v>
+      </c>
+      <c r="O261" t="str">
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/99240040687.jpg</v>
+      </c>
+      <c r="P261" t="str">
+        <v>7/8/2026, 3:46:42 pm</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262">
+        <v>261</v>
+      </c>
+      <c r="B262" t="str">
+        <v>V MALLIKARJUNA</v>
+      </c>
+      <c r="C262" t="str">
+        <v>99240040181</v>
+      </c>
+      <c r="D262" t="str">
+        <v>154154599395</v>
+      </c>
+      <c r="E262" t="str">
+        <v>99240040181@klu.ac.in</v>
+      </c>
+      <c r="F262" t="str">
+        <v>9876543210</v>
+      </c>
+      <c r="G262" t="str">
+        <v>CSE</v>
+      </c>
+      <c r="H262" t="str">
+        <v>III Year</v>
+      </c>
+      <c r="I262" t="str">
+        <v>24S18</v>
+      </c>
+      <c r="J262" t="str">
+        <v>Hosteller</v>
+      </c>
+      <c r="K262" t="str">
+        <v>Approved</v>
+      </c>
+      <c r="L262" t="str">
+        <v>Registered</v>
+      </c>
+      <c r="M262" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="N262" t="str">
+        <v>claim-group-3/payment-screenshots/99240040181</v>
+      </c>
+      <c r="O262" t="str">
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/99240040181.jpg</v>
+      </c>
+      <c r="P262" t="str">
+        <v>7/8/2026, 3:46:43 pm</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263">
+        <v>262</v>
+      </c>
+      <c r="B263" t="str">
+        <v>BOMMADI ISHANT SRI</v>
+      </c>
+      <c r="C263" t="str">
+        <v>99240040405</v>
+      </c>
+      <c r="D263" t="str">
+        <v>531300933205</v>
+      </c>
+      <c r="E263" t="str">
+        <v>99240040405@klu.ac.in</v>
+      </c>
+      <c r="F263" t="str">
+        <v>9876543210</v>
+      </c>
+      <c r="G263" t="str">
+        <v>CSE</v>
+      </c>
+      <c r="H263" t="str">
+        <v>III Year</v>
+      </c>
+      <c r="I263" t="str">
+        <v>24S04</v>
+      </c>
+      <c r="J263" t="str">
+        <v>Hosteller</v>
+      </c>
+      <c r="K263" t="str">
+        <v>Approved</v>
+      </c>
+      <c r="L263" t="str">
+        <v>Registered</v>
+      </c>
+      <c r="M263" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="N263" t="str">
+        <v>claim-group-3/payment-screenshots/99240040405</v>
+      </c>
+      <c r="O263" t="str">
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/99240040405.jpg</v>
+      </c>
+      <c r="P263" t="str">
+        <v>7/8/2026, 3:46:43 pm</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P260"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P263"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 17 offline registrants, fix multi-device attendance sync, and create /attend volunteer portal
</commit_message>
<xml_diff>
--- a/CSI_KARE_ML_Pipeline_All_Registrations_Clean.xlsx
+++ b/CSI_KARE_ML_Pipeline_All_Registrations_Clean.xlsx
@@ -397,25 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P263"/>
-  <cols>
-    <col min="1" max="1" width="16.83203125" customWidth="1"/>
-    <col min="2" max="2" width="16.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="27.83203125" customWidth="1"/>
-    <col min="5" max="5" width="16.83203125" customWidth="1"/>
-    <col min="6" max="6" width="16.83203125" customWidth="1"/>
-    <col min="7" max="7" width="16.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="16.83203125" customWidth="1"/>
-    <col min="10" max="10" width="19.83203125" customWidth="1"/>
-    <col min="11" max="11" width="17.83203125" customWidth="1"/>
-    <col min="12" max="12" width="22.83203125" customWidth="1"/>
-    <col min="13" max="13" width="19.83203125" customWidth="1"/>
-    <col min="14" max="14" width="23.83203125" customWidth="1"/>
-    <col min="15" max="15" width="25.83203125" customWidth="1"/>
-    <col min="16" max="16" width="20.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:P280"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -13567,9 +13549,859 @@
         <v>7/8/2026, 3:46:43 pm</v>
       </c>
     </row>
+    <row r="264">
+      <c r="A264">
+        <v>263</v>
+      </c>
+      <c r="B264" t="str">
+        <v>KUNCHAM LAKSHMI NARASIMHA REDDY</v>
+      </c>
+      <c r="C264" t="str">
+        <v>99230040631</v>
+      </c>
+      <c r="D264" t="str">
+        <v>OFFLINE_208933000263</v>
+      </c>
+      <c r="E264" t="str">
+        <v>99230040631@klu.ac.in</v>
+      </c>
+      <c r="F264" t="str">
+        <v>9876543210</v>
+      </c>
+      <c r="G264" t="str">
+        <v>CSE</v>
+      </c>
+      <c r="H264" t="str">
+        <v>IV Year</v>
+      </c>
+      <c r="I264" t="str">
+        <v>S08</v>
+      </c>
+      <c r="J264" t="str">
+        <v>Day Scholar</v>
+      </c>
+      <c r="K264" t="str">
+        <v>Approved</v>
+      </c>
+      <c r="L264" t="str">
+        <v>Registered</v>
+      </c>
+      <c r="M264" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="N264" t="str">
+        <v>claim-group-3/payment-screenshots/99230040631</v>
+      </c>
+      <c r="O264" t="str">
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/99230040631.jpg</v>
+      </c>
+      <c r="P264" t="str">
+        <v>8/8/2026, 12:00:00 pm</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265">
+        <v>264</v>
+      </c>
+      <c r="B265" t="str">
+        <v>DADIYALA HITHESH</v>
+      </c>
+      <c r="C265" t="str">
+        <v>99230040905</v>
+      </c>
+      <c r="D265" t="str">
+        <v>OFFLINE_208933000264</v>
+      </c>
+      <c r="E265" t="str">
+        <v>99230040905@klu.ac.in</v>
+      </c>
+      <c r="F265" t="str">
+        <v>9876543210</v>
+      </c>
+      <c r="G265" t="str">
+        <v>CSE</v>
+      </c>
+      <c r="H265" t="str">
+        <v>IV Year</v>
+      </c>
+      <c r="I265" t="str">
+        <v>S08</v>
+      </c>
+      <c r="J265" t="str">
+        <v>Day Scholar</v>
+      </c>
+      <c r="K265" t="str">
+        <v>Approved</v>
+      </c>
+      <c r="L265" t="str">
+        <v>Registered</v>
+      </c>
+      <c r="M265" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="N265" t="str">
+        <v>claim-group-3/payment-screenshots/99230040905</v>
+      </c>
+      <c r="O265" t="str">
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/99230040905.jpg</v>
+      </c>
+      <c r="P265" t="str">
+        <v>8/8/2026, 12:00:00 pm</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266">
+        <v>265</v>
+      </c>
+      <c r="B266" t="str">
+        <v>KANNA PRANAVI SRINIVAS</v>
+      </c>
+      <c r="C266" t="str">
+        <v>99230040932</v>
+      </c>
+      <c r="D266" t="str">
+        <v>OFFLINE_208933000265</v>
+      </c>
+      <c r="E266" t="str">
+        <v>99230040932@klu.ac.in</v>
+      </c>
+      <c r="F266" t="str">
+        <v>9876543210</v>
+      </c>
+      <c r="G266" t="str">
+        <v>CSE</v>
+      </c>
+      <c r="H266" t="str">
+        <v>IV Year</v>
+      </c>
+      <c r="I266" t="str">
+        <v>S08</v>
+      </c>
+      <c r="J266" t="str">
+        <v>Day Scholar</v>
+      </c>
+      <c r="K266" t="str">
+        <v>Approved</v>
+      </c>
+      <c r="L266" t="str">
+        <v>Registered</v>
+      </c>
+      <c r="M266" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="N266" t="str">
+        <v>claim-group-3/payment-screenshots/99230040932</v>
+      </c>
+      <c r="O266" t="str">
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/99230040932.jpg</v>
+      </c>
+      <c r="P266" t="str">
+        <v>8/8/2026, 12:00:00 pm</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267">
+        <v>266</v>
+      </c>
+      <c r="B267" t="str">
+        <v>P. TEJA SIMHA REDDY</v>
+      </c>
+      <c r="C267" t="str">
+        <v>9923005316</v>
+      </c>
+      <c r="D267" t="str">
+        <v>OFFLINE_208933000266</v>
+      </c>
+      <c r="E267" t="str">
+        <v>9923005316@klu.ac.in</v>
+      </c>
+      <c r="F267" t="str">
+        <v>9160740077</v>
+      </c>
+      <c r="G267" t="str">
+        <v>ECE</v>
+      </c>
+      <c r="H267" t="str">
+        <v>IV Year</v>
+      </c>
+      <c r="I267" t="str">
+        <v>ECE-A</v>
+      </c>
+      <c r="J267" t="str">
+        <v>Hosteller</v>
+      </c>
+      <c r="K267" t="str">
+        <v>Approved</v>
+      </c>
+      <c r="L267" t="str">
+        <v>Registered</v>
+      </c>
+      <c r="M267" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="N267" t="str">
+        <v>claim-group-3/payment-screenshots/9923005316</v>
+      </c>
+      <c r="O267" t="str">
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/9923005316.jpg</v>
+      </c>
+      <c r="P267" t="str">
+        <v>8/8/2026, 12:00:00 pm</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268">
+        <v>267</v>
+      </c>
+      <c r="B268" t="str">
+        <v>K. GURU TEJA</v>
+      </c>
+      <c r="C268" t="str">
+        <v>9923005320</v>
+      </c>
+      <c r="D268" t="str">
+        <v>OFFLINE_208933000267</v>
+      </c>
+      <c r="E268" t="str">
+        <v>9923005320@klu.ac.in</v>
+      </c>
+      <c r="F268" t="str">
+        <v>9347735134</v>
+      </c>
+      <c r="G268" t="str">
+        <v>ECE</v>
+      </c>
+      <c r="H268" t="str">
+        <v>IV Year</v>
+      </c>
+      <c r="I268" t="str">
+        <v>ECE-A</v>
+      </c>
+      <c r="J268" t="str">
+        <v>Day Scholar</v>
+      </c>
+      <c r="K268" t="str">
+        <v>Approved</v>
+      </c>
+      <c r="L268" t="str">
+        <v>Registered</v>
+      </c>
+      <c r="M268" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="N268" t="str">
+        <v>claim-group-3/payment-screenshots/9923005320</v>
+      </c>
+      <c r="O268" t="str">
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/9923005320.jpg</v>
+      </c>
+      <c r="P268" t="str">
+        <v>8/8/2026, 12:00:00 pm</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269">
+        <v>268</v>
+      </c>
+      <c r="B269" t="str">
+        <v>D. ANJANEYULU</v>
+      </c>
+      <c r="C269" t="str">
+        <v>9923005074</v>
+      </c>
+      <c r="D269" t="str">
+        <v>OFFLINE_208933000268</v>
+      </c>
+      <c r="E269" t="str">
+        <v>9923005074@klu.ac.in</v>
+      </c>
+      <c r="F269" t="str">
+        <v>9121540275</v>
+      </c>
+      <c r="G269" t="str">
+        <v>ECE</v>
+      </c>
+      <c r="H269" t="str">
+        <v>IV Year</v>
+      </c>
+      <c r="I269" t="str">
+        <v>ECE-A</v>
+      </c>
+      <c r="J269" t="str">
+        <v>Day Scholar</v>
+      </c>
+      <c r="K269" t="str">
+        <v>Approved</v>
+      </c>
+      <c r="L269" t="str">
+        <v>Registered</v>
+      </c>
+      <c r="M269" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="N269" t="str">
+        <v>claim-group-3/payment-screenshots/9923005074</v>
+      </c>
+      <c r="O269" t="str">
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/9923005074.jpg</v>
+      </c>
+      <c r="P269" t="str">
+        <v>8/8/2026, 12:00:00 pm</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270">
+        <v>269</v>
+      </c>
+      <c r="B270" t="str">
+        <v>AYULURI SOMANADH MADHAVA REDDY</v>
+      </c>
+      <c r="C270" t="str">
+        <v>99230041030</v>
+      </c>
+      <c r="D270" t="str">
+        <v>OFFLINE_208933000269</v>
+      </c>
+      <c r="E270" t="str">
+        <v>99230041030@klu.ac.in</v>
+      </c>
+      <c r="F270" t="str">
+        <v>9666347772</v>
+      </c>
+      <c r="G270" t="str">
+        <v>CSE</v>
+      </c>
+      <c r="H270" t="str">
+        <v>IV Year</v>
+      </c>
+      <c r="I270" t="str">
+        <v>23S13</v>
+      </c>
+      <c r="J270" t="str">
+        <v>Day Scholar</v>
+      </c>
+      <c r="K270" t="str">
+        <v>Approved</v>
+      </c>
+      <c r="L270" t="str">
+        <v>Registered</v>
+      </c>
+      <c r="M270" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="N270" t="str">
+        <v>claim-group-3/payment-screenshots/99230041030</v>
+      </c>
+      <c r="O270" t="str">
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/99230041030.jpg</v>
+      </c>
+      <c r="P270" t="str">
+        <v>8/8/2026, 12:00:00 pm</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271">
+        <v>270</v>
+      </c>
+      <c r="B271" t="str">
+        <v>G. HEMALATHA</v>
+      </c>
+      <c r="C271" t="str">
+        <v>99230040300</v>
+      </c>
+      <c r="D271" t="str">
+        <v>OFFLINE_208933000270</v>
+      </c>
+      <c r="E271" t="str">
+        <v>99230040300@klu.ac.in</v>
+      </c>
+      <c r="F271" t="str">
+        <v>9346383312</v>
+      </c>
+      <c r="G271" t="str">
+        <v>CSE</v>
+      </c>
+      <c r="H271" t="str">
+        <v>IV Year</v>
+      </c>
+      <c r="I271" t="str">
+        <v>S04</v>
+      </c>
+      <c r="J271" t="str">
+        <v>Hosteller</v>
+      </c>
+      <c r="K271" t="str">
+        <v>Approved</v>
+      </c>
+      <c r="L271" t="str">
+        <v>Registered</v>
+      </c>
+      <c r="M271" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="N271" t="str">
+        <v>claim-group-3/payment-screenshots/99230040300</v>
+      </c>
+      <c r="O271" t="str">
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/99230040300.jpg</v>
+      </c>
+      <c r="P271" t="str">
+        <v>8/8/2026, 12:00:00 pm</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272">
+        <v>271</v>
+      </c>
+      <c r="B272" t="str">
+        <v>SHAIK MOHAMMED TAHEER</v>
+      </c>
+      <c r="C272" t="str">
+        <v>99240040767</v>
+      </c>
+      <c r="D272" t="str">
+        <v>OFFLINE_208933000271</v>
+      </c>
+      <c r="E272" t="str">
+        <v>99240040767@klu.ac.in</v>
+      </c>
+      <c r="F272" t="str">
+        <v>9440337129</v>
+      </c>
+      <c r="G272" t="str">
+        <v>CSE</v>
+      </c>
+      <c r="H272" t="str">
+        <v>III Year</v>
+      </c>
+      <c r="I272" t="str">
+        <v>24S09</v>
+      </c>
+      <c r="J272" t="str">
+        <v>Day Scholar</v>
+      </c>
+      <c r="K272" t="str">
+        <v>Approved</v>
+      </c>
+      <c r="L272" t="str">
+        <v>Registered</v>
+      </c>
+      <c r="M272" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="N272" t="str">
+        <v>claim-group-3/payment-screenshots/99240040767</v>
+      </c>
+      <c r="O272" t="str">
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/99240040767.jpg</v>
+      </c>
+      <c r="P272" t="str">
+        <v>8/8/2026, 12:00:00 pm</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273">
+        <v>272</v>
+      </c>
+      <c r="B273" t="str">
+        <v>SEELAM BHANU PRAKASH REDDY</v>
+      </c>
+      <c r="C273" t="str">
+        <v>99240040783</v>
+      </c>
+      <c r="D273" t="str">
+        <v>OFFLINE_208933000272</v>
+      </c>
+      <c r="E273" t="str">
+        <v>99240040783@klu.ac.in</v>
+      </c>
+      <c r="F273" t="str">
+        <v>6302684215</v>
+      </c>
+      <c r="G273" t="str">
+        <v>CSE</v>
+      </c>
+      <c r="H273" t="str">
+        <v>III Year</v>
+      </c>
+      <c r="I273" t="str">
+        <v>24S09</v>
+      </c>
+      <c r="J273" t="str">
+        <v>Day Scholar</v>
+      </c>
+      <c r="K273" t="str">
+        <v>Approved</v>
+      </c>
+      <c r="L273" t="str">
+        <v>Registered</v>
+      </c>
+      <c r="M273" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="N273" t="str">
+        <v>claim-group-3/payment-screenshots/99240040783</v>
+      </c>
+      <c r="O273" t="str">
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/99240040783.jpg</v>
+      </c>
+      <c r="P273" t="str">
+        <v>8/8/2026, 12:00:00 pm</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274">
+        <v>273</v>
+      </c>
+      <c r="B274" t="str">
+        <v>DEGA RAKESH</v>
+      </c>
+      <c r="C274" t="str">
+        <v>99240040777</v>
+      </c>
+      <c r="D274" t="str">
+        <v>OFFLINE_208933000273</v>
+      </c>
+      <c r="E274" t="str">
+        <v>99240040777@klu.ac.in</v>
+      </c>
+      <c r="F274" t="str">
+        <v>8374248157</v>
+      </c>
+      <c r="G274" t="str">
+        <v>CSE</v>
+      </c>
+      <c r="H274" t="str">
+        <v>III Year</v>
+      </c>
+      <c r="I274" t="str">
+        <v>24S09</v>
+      </c>
+      <c r="J274" t="str">
+        <v>Hosteller</v>
+      </c>
+      <c r="K274" t="str">
+        <v>Approved</v>
+      </c>
+      <c r="L274" t="str">
+        <v>Registered</v>
+      </c>
+      <c r="M274" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="N274" t="str">
+        <v>claim-group-3/payment-screenshots/99240040777</v>
+      </c>
+      <c r="O274" t="str">
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/99240040777.jpg</v>
+      </c>
+      <c r="P274" t="str">
+        <v>8/8/2026, 12:00:00 pm</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275">
+        <v>274</v>
+      </c>
+      <c r="B275" t="str">
+        <v>DOKKA OMKAR</v>
+      </c>
+      <c r="C275" t="str">
+        <v>9924005238</v>
+      </c>
+      <c r="D275" t="str">
+        <v>OFFLINE_208933000274</v>
+      </c>
+      <c r="E275" t="str">
+        <v>9924005238@klu.ac.in</v>
+      </c>
+      <c r="F275" t="str">
+        <v>9876543210</v>
+      </c>
+      <c r="G275" t="str">
+        <v>ECE</v>
+      </c>
+      <c r="H275" t="str">
+        <v>III Year</v>
+      </c>
+      <c r="I275" t="str">
+        <v>ECE-A</v>
+      </c>
+      <c r="J275" t="str">
+        <v>Day Scholar</v>
+      </c>
+      <c r="K275" t="str">
+        <v>Approved</v>
+      </c>
+      <c r="L275" t="str">
+        <v>Registered</v>
+      </c>
+      <c r="M275" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="N275" t="str">
+        <v>claim-group-3/payment-screenshots/9924005238</v>
+      </c>
+      <c r="O275" t="str">
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/9924005238.jpg</v>
+      </c>
+      <c r="P275" t="str">
+        <v>8/8/2026, 12:00:00 pm</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276">
+        <v>275</v>
+      </c>
+      <c r="B276" t="str">
+        <v>MODDURU LALITHA</v>
+      </c>
+      <c r="C276" t="str">
+        <v>9924005108</v>
+      </c>
+      <c r="D276" t="str">
+        <v>OFFLINE_208933000275</v>
+      </c>
+      <c r="E276" t="str">
+        <v>9924005108@klu.ac.in</v>
+      </c>
+      <c r="F276" t="str">
+        <v>9876543210</v>
+      </c>
+      <c r="G276" t="str">
+        <v>ECE</v>
+      </c>
+      <c r="H276" t="str">
+        <v>III Year</v>
+      </c>
+      <c r="I276" t="str">
+        <v>F</v>
+      </c>
+      <c r="J276" t="str">
+        <v>Hosteller</v>
+      </c>
+      <c r="K276" t="str">
+        <v>Approved</v>
+      </c>
+      <c r="L276" t="str">
+        <v>Registered</v>
+      </c>
+      <c r="M276" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="N276" t="str">
+        <v>claim-group-3/payment-screenshots/9924005108</v>
+      </c>
+      <c r="O276" t="str">
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/9924005108.jpg</v>
+      </c>
+      <c r="P276" t="str">
+        <v>8/8/2026, 12:00:00 pm</v>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277">
+        <v>276</v>
+      </c>
+      <c r="B277" t="str">
+        <v>KALLAMADI VENUMADHAV REDDY</v>
+      </c>
+      <c r="C277" t="str">
+        <v>99250040348</v>
+      </c>
+      <c r="D277" t="str">
+        <v>OFFLINE_208933000276</v>
+      </c>
+      <c r="E277" t="str">
+        <v>99250040348@klu.ac.in</v>
+      </c>
+      <c r="F277" t="str">
+        <v>8919339618</v>
+      </c>
+      <c r="G277" t="str">
+        <v>CSE</v>
+      </c>
+      <c r="H277" t="str">
+        <v>II Year</v>
+      </c>
+      <c r="I277" t="str">
+        <v>25S04</v>
+      </c>
+      <c r="J277" t="str">
+        <v>Day Scholar</v>
+      </c>
+      <c r="K277" t="str">
+        <v>Approved</v>
+      </c>
+      <c r="L277" t="str">
+        <v>Registered</v>
+      </c>
+      <c r="M277" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="N277" t="str">
+        <v>claim-group-3/payment-screenshots/99250040348</v>
+      </c>
+      <c r="O277" t="str">
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/99250040348.jpg</v>
+      </c>
+      <c r="P277" t="str">
+        <v>8/8/2026, 12:00:00 pm</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278">
+        <v>277</v>
+      </c>
+      <c r="B278" t="str">
+        <v>MACHA PUNEEETH RAM</v>
+      </c>
+      <c r="C278" t="str">
+        <v>99250040322</v>
+      </c>
+      <c r="D278" t="str">
+        <v>OFFLINE_208933000277</v>
+      </c>
+      <c r="E278" t="str">
+        <v>99250040322@klu.ac.in</v>
+      </c>
+      <c r="F278" t="str">
+        <v>9494324718</v>
+      </c>
+      <c r="G278" t="str">
+        <v>CSE</v>
+      </c>
+      <c r="H278" t="str">
+        <v>II Year</v>
+      </c>
+      <c r="I278" t="str">
+        <v>25S04</v>
+      </c>
+      <c r="J278" t="str">
+        <v>Day Scholar</v>
+      </c>
+      <c r="K278" t="str">
+        <v>Approved</v>
+      </c>
+      <c r="L278" t="str">
+        <v>Registered</v>
+      </c>
+      <c r="M278" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="N278" t="str">
+        <v>claim-group-3/payment-screenshots/99250040322</v>
+      </c>
+      <c r="O278" t="str">
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/99250040322.jpg</v>
+      </c>
+      <c r="P278" t="str">
+        <v>8/8/2026, 12:00:00 pm</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279">
+        <v>278</v>
+      </c>
+      <c r="B279" t="str">
+        <v>G. MANOJ</v>
+      </c>
+      <c r="C279" t="str">
+        <v>99250040229</v>
+      </c>
+      <c r="D279" t="str">
+        <v>OFFLINE_208933000278</v>
+      </c>
+      <c r="E279" t="str">
+        <v>99250040229@klu.ac.in</v>
+      </c>
+      <c r="F279" t="str">
+        <v>9502847774</v>
+      </c>
+      <c r="G279" t="str">
+        <v>CSE (AI &amp; ML)</v>
+      </c>
+      <c r="H279" t="str">
+        <v>II Year</v>
+      </c>
+      <c r="I279" t="str">
+        <v>25S03</v>
+      </c>
+      <c r="J279" t="str">
+        <v>Hosteller</v>
+      </c>
+      <c r="K279" t="str">
+        <v>Approved</v>
+      </c>
+      <c r="L279" t="str">
+        <v>Registered</v>
+      </c>
+      <c r="M279" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="N279" t="str">
+        <v>claim-group-3/payment-screenshots/99250040229</v>
+      </c>
+      <c r="O279" t="str">
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/99250040229.jpg</v>
+      </c>
+      <c r="P279" t="str">
+        <v>8/8/2026, 12:00:00 pm</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280">
+        <v>279</v>
+      </c>
+      <c r="B280" t="str">
+        <v>IRALA HEMANTH</v>
+      </c>
+      <c r="C280" t="str">
+        <v>99250040392</v>
+      </c>
+      <c r="D280" t="str">
+        <v>OFFLINE_208933000279</v>
+      </c>
+      <c r="E280" t="str">
+        <v>99250040392@klu.ac.in</v>
+      </c>
+      <c r="F280" t="str">
+        <v>8463982154</v>
+      </c>
+      <c r="G280" t="str">
+        <v>CSE (AI &amp; ML)</v>
+      </c>
+      <c r="H280" t="str">
+        <v>II Year</v>
+      </c>
+      <c r="I280" t="str">
+        <v>25S05</v>
+      </c>
+      <c r="J280" t="str">
+        <v>Hosteller</v>
+      </c>
+      <c r="K280" t="str">
+        <v>Approved</v>
+      </c>
+      <c r="L280" t="str">
+        <v>Registered</v>
+      </c>
+      <c r="M280" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="N280" t="str">
+        <v>claim-group-3/payment-screenshots/99250040392</v>
+      </c>
+      <c r="O280" t="str">
+        <v>https://res.cloudinary.com/dmst2wexn/image/upload/v1786076854/claim-group-3/payment-screenshots/99250040392.jpg</v>
+      </c>
+      <c r="P280" t="str">
+        <v>8/8/2026, 12:00:00 pm</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P263"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P280"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>